<commit_message>
forest land , plot dist etc
</commit_message>
<xml_diff>
--- a/uploads/excels/LIMS_Test_Pvt_land_Data_format_24.03.26_(1)_(3)_(1).xlsx
+++ b/uploads/excels/LIMS_Test_Pvt_land_Data_format_24.03.26_(1)_(3)_(1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maasuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2607BCDD-1022-40C4-9FF1-217FC3438FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E720A31-B77E-494A-B8C0-08B3E617EC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="308">
   <si>
     <t>SES Survey No.</t>
   </si>
@@ -1600,6 +1600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:CK35"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1938,7 +1939,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:89" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:89" ht="54.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -2195,7 +2196,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="3" spans="1:89" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:89" ht="62.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -2447,7 +2448,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="4" spans="1:89" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:89" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -2965,7 +2966,9 @@
       <c r="M6" s="11">
         <v>172</v>
       </c>
-      <c r="N6" s="12"/>
+      <c r="N6" s="12" t="s">
+        <v>128</v>
+      </c>
       <c r="O6" s="11" t="s">
         <v>139</v>
       </c>
@@ -3182,7 +3185,9 @@
       <c r="M7" s="11">
         <v>172</v>
       </c>
-      <c r="N7" s="12"/>
+      <c r="N7" s="12" t="s">
+        <v>128</v>
+      </c>
       <c r="O7" s="11" t="s">
         <v>139</v>
       </c>
@@ -3369,7 +3374,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="8" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -3475,7 +3480,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -3577,7 +3582,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="10" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -3695,7 +3700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -3800,7 +3805,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="12" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -3904,7 +3909,7 @@
       <c r="AQ12" s="25"/>
       <c r="AR12" s="25"/>
     </row>
-    <row r="13" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -4004,7 +4009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:89" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:89" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -4112,7 +4117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:89" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:89" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -4306,7 +4311,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="16" spans="1:89" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:89" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>15</v>
       </c>
@@ -4481,7 +4486,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="17" spans="1:62" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:62" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>16</v>
       </c>
@@ -4586,7 +4591,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="18" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -4691,7 +4696,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="19" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>18</v>
       </c>
@@ -4796,7 +4801,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="20" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -4901,7 +4906,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>20</v>
       </c>
@@ -5006,7 +5011,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="22" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>21</v>
       </c>
@@ -5111,7 +5116,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="23" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>22</v>
       </c>
@@ -5216,7 +5221,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="24" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <v>23</v>
       </c>
@@ -5321,7 +5326,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="25" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>24</v>
       </c>
@@ -5425,7 +5430,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="26" spans="1:62" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:62" ht="75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>25</v>
       </c>
@@ -5531,7 +5536,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>26</v>
       </c>
@@ -5622,7 +5627,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="28" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <v>27</v>
       </c>
@@ -5717,7 +5722,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="29" spans="1:62" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:62" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>28</v>
       </c>
@@ -5819,7 +5824,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="30" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:62" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>29</v>
       </c>
@@ -5921,7 +5926,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="31" spans="1:62" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:62" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>30</v>
       </c>
@@ -6027,7 +6032,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="32" spans="1:62" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:62" ht="110.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <v>31</v>
       </c>
@@ -6110,6 +6115,13 @@
       <c r="R35" s="38"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:CK32" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="12">
+      <filters>
+        <filter val="172"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="M1">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>